<commit_message>
Biagolini Blanks to NA
Find-replaced whole empty cells with "NA"
</commit_message>
<xml_diff>
--- a/Source Data Process_CB/Biagolini_SuppTable1.xlsx
+++ b/Source Data Process_CB/Biagolini_SuppTable1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/kate/Desktop/CooperativeBreedingEvolution/Source Data Process_CB/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FB3E1A7C-EF95-4E47-AB47-A620B9306F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E8DBF515-2F65-3A48-8F3D-A0DEFB313D9F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="1160" yWindow="660" windowWidth="28040" windowHeight="17280" xr2:uid="{10AD7567-51C1-244C-9C49-3C4EE696AFD4}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1741" uniqueCount="959">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2530" uniqueCount="959">
   <si>
     <t>OR</t>
   </si>
@@ -3567,10 +3567,18 @@
       <c r="I3" s="7">
         <v>44</v>
       </c>
-      <c r="J3" s="8"/>
-      <c r="K3" s="8"/>
-      <c r="L3" s="8"/>
-      <c r="M3" s="8"/>
+      <c r="J3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L3" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M3" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N3" s="5" t="s">
         <v>18</v>
       </c>
@@ -3647,10 +3655,18 @@
       <c r="I5" s="7">
         <v>19</v>
       </c>
-      <c r="J5" s="8"/>
-      <c r="K5" s="8"/>
-      <c r="L5" s="8"/>
-      <c r="M5" s="8"/>
+      <c r="J5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L5" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M5" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N5" s="5" t="s">
         <v>23</v>
       </c>
@@ -3683,10 +3699,18 @@
       <c r="I6" s="7">
         <v>40</v>
       </c>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8"/>
+      <c r="J6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N6" s="5" t="s">
         <v>25</v>
       </c>
@@ -3719,10 +3743,18 @@
       <c r="I7" s="7">
         <v>25</v>
       </c>
-      <c r="J7" s="8"/>
-      <c r="K7" s="8"/>
-      <c r="L7" s="8"/>
-      <c r="M7" s="8"/>
+      <c r="J7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L7" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M7" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N7" s="5" t="s">
         <v>28</v>
       </c>
@@ -3755,10 +3787,18 @@
       <c r="I8" s="7">
         <v>23</v>
       </c>
-      <c r="J8" s="8"/>
-      <c r="K8" s="8"/>
-      <c r="L8" s="8"/>
-      <c r="M8" s="8"/>
+      <c r="J8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N8" s="5" t="s">
         <v>30</v>
       </c>
@@ -3791,10 +3831,18 @@
       <c r="I9" s="7">
         <v>24</v>
       </c>
-      <c r="J9" s="8"/>
-      <c r="K9" s="8"/>
-      <c r="L9" s="8"/>
-      <c r="M9" s="8"/>
+      <c r="J9" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K9" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L9" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M9" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N9" s="5" t="s">
         <v>30</v>
       </c>
@@ -3827,10 +3875,18 @@
       <c r="I10" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J10" s="7"/>
-      <c r="K10" s="9"/>
-      <c r="L10" s="9"/>
-      <c r="M10" s="9"/>
+      <c r="J10" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="L10" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="M10" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="N10" s="5" t="s">
         <v>33</v>
       </c>
@@ -3863,10 +3919,18 @@
       <c r="I11" s="7">
         <v>42</v>
       </c>
-      <c r="J11" s="8"/>
-      <c r="K11" s="8"/>
-      <c r="L11" s="8"/>
-      <c r="M11" s="8"/>
+      <c r="J11" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K11" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L11" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M11" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N11" s="5" t="s">
         <v>35</v>
       </c>
@@ -3899,10 +3963,18 @@
       <c r="I12" s="7">
         <v>72</v>
       </c>
-      <c r="J12" s="8"/>
-      <c r="K12" s="8"/>
-      <c r="L12" s="8"/>
-      <c r="M12" s="8"/>
+      <c r="J12" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K12" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L12" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M12" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N12" s="5" t="s">
         <v>37</v>
       </c>
@@ -3935,10 +4007,18 @@
       <c r="I13" s="7">
         <v>85</v>
       </c>
-      <c r="J13" s="8"/>
-      <c r="K13" s="8"/>
-      <c r="L13" s="8"/>
-      <c r="M13" s="8"/>
+      <c r="J13" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K13" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L13" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M13" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N13" s="5" t="s">
         <v>39</v>
       </c>
@@ -3971,10 +4051,18 @@
       <c r="I14" s="7">
         <v>4</v>
       </c>
-      <c r="J14" s="8"/>
-      <c r="K14" s="8"/>
-      <c r="L14" s="8"/>
-      <c r="M14" s="8"/>
+      <c r="J14" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K14" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L14" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M14" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N14" s="5" t="s">
         <v>41</v>
       </c>
@@ -4007,10 +4095,18 @@
       <c r="I15" s="7">
         <v>38</v>
       </c>
-      <c r="J15" s="8"/>
-      <c r="K15" s="8"/>
-      <c r="L15" s="8"/>
-      <c r="M15" s="8"/>
+      <c r="J15" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K15" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L15" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M15" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N15" s="5" t="s">
         <v>44</v>
       </c>
@@ -4087,10 +4183,18 @@
       <c r="I17" s="7">
         <v>4</v>
       </c>
-      <c r="J17" s="8"/>
-      <c r="K17" s="8"/>
-      <c r="L17" s="8"/>
-      <c r="M17" s="8"/>
+      <c r="J17" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K17" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L17" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M17" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N17" s="5" t="s">
         <v>51</v>
       </c>
@@ -4123,10 +4227,18 @@
       <c r="I18" s="7">
         <v>16</v>
       </c>
-      <c r="J18" s="8"/>
-      <c r="K18" s="8"/>
-      <c r="L18" s="8"/>
-      <c r="M18" s="8"/>
+      <c r="J18" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K18" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L18" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M18" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N18" s="5" t="s">
         <v>54</v>
       </c>
@@ -4159,10 +4271,18 @@
       <c r="I19" s="7">
         <v>88</v>
       </c>
-      <c r="J19" s="8"/>
-      <c r="K19" s="8"/>
-      <c r="L19" s="8"/>
-      <c r="M19" s="8"/>
+      <c r="J19" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K19" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L19" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M19" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N19" s="5" t="s">
         <v>57</v>
       </c>
@@ -4195,10 +4315,18 @@
       <c r="I20" s="7">
         <v>32</v>
       </c>
-      <c r="J20" s="8"/>
-      <c r="K20" s="8"/>
-      <c r="L20" s="8"/>
-      <c r="M20" s="8"/>
+      <c r="J20" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K20" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L20" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M20" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N20" s="5" t="s">
         <v>59</v>
       </c>
@@ -4231,10 +4359,18 @@
       <c r="I21" s="7">
         <v>38</v>
       </c>
-      <c r="J21" s="8"/>
-      <c r="K21" s="8"/>
-      <c r="L21" s="8"/>
-      <c r="M21" s="8"/>
+      <c r="J21" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K21" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L21" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M21" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N21" s="5" t="s">
         <v>61</v>
       </c>
@@ -4267,10 +4403,18 @@
       <c r="I22" s="7">
         <v>77</v>
       </c>
-      <c r="J22" s="8"/>
-      <c r="K22" s="8"/>
-      <c r="L22" s="8"/>
-      <c r="M22" s="8"/>
+      <c r="J22" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K22" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L22" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M22" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N22" s="5" t="s">
         <v>63</v>
       </c>
@@ -4303,10 +4447,18 @@
       <c r="I23" s="7">
         <v>27</v>
       </c>
-      <c r="J23" s="8"/>
-      <c r="K23" s="8"/>
-      <c r="L23" s="8"/>
-      <c r="M23" s="8"/>
+      <c r="J23" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K23" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L23" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M23" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N23" s="5" t="s">
         <v>65</v>
       </c>
@@ -4383,10 +4535,18 @@
       <c r="I25" s="7">
         <v>24</v>
       </c>
-      <c r="J25" s="8"/>
-      <c r="K25" s="8"/>
-      <c r="L25" s="8"/>
-      <c r="M25" s="8"/>
+      <c r="J25" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K25" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L25" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M25" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N25" s="5" t="s">
         <v>71</v>
       </c>
@@ -4463,10 +4623,18 @@
       <c r="I27" s="7">
         <v>20</v>
       </c>
-      <c r="J27" s="8"/>
-      <c r="K27" s="8"/>
-      <c r="L27" s="8"/>
-      <c r="M27" s="8"/>
+      <c r="J27" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K27" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L27" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M27" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N27" s="5" t="s">
         <v>76</v>
       </c>
@@ -4499,10 +4667,18 @@
       <c r="I28" s="7">
         <v>26</v>
       </c>
-      <c r="J28" s="7"/>
-      <c r="K28" s="9"/>
-      <c r="L28" s="9"/>
-      <c r="M28" s="9"/>
+      <c r="J28" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K28" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="L28" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="M28" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="N28" s="5" t="s">
         <v>79</v>
       </c>
@@ -4623,10 +4799,18 @@
       <c r="I31" s="7">
         <v>30</v>
       </c>
-      <c r="J31" s="8"/>
-      <c r="K31" s="8"/>
-      <c r="L31" s="8"/>
-      <c r="M31" s="8"/>
+      <c r="J31" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K31" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L31" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M31" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N31" s="5" t="s">
         <v>88</v>
       </c>
@@ -4659,10 +4843,18 @@
       <c r="I32" s="7">
         <v>11</v>
       </c>
-      <c r="J32" s="8"/>
-      <c r="K32" s="8"/>
-      <c r="L32" s="8"/>
-      <c r="M32" s="8"/>
+      <c r="J32" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K32" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L32" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M32" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N32" s="5" t="s">
         <v>90</v>
       </c>
@@ -4695,10 +4887,18 @@
       <c r="I33" s="7">
         <v>24</v>
       </c>
-      <c r="J33" s="8"/>
-      <c r="K33" s="8"/>
-      <c r="L33" s="8"/>
-      <c r="M33" s="8"/>
+      <c r="J33" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K33" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L33" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M33" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N33" s="5" t="s">
         <v>92</v>
       </c>
@@ -4731,10 +4931,18 @@
       <c r="I34" s="7">
         <v>22</v>
       </c>
-      <c r="J34" s="8"/>
-      <c r="K34" s="8"/>
-      <c r="L34" s="8"/>
-      <c r="M34" s="8"/>
+      <c r="J34" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K34" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L34" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M34" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N34" s="5" t="s">
         <v>94</v>
       </c>
@@ -4767,10 +4975,18 @@
       <c r="I35" s="7">
         <v>30</v>
       </c>
-      <c r="J35" s="8"/>
-      <c r="K35" s="8"/>
-      <c r="L35" s="8"/>
-      <c r="M35" s="8"/>
+      <c r="J35" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K35" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L35" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M35" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N35" s="5" t="s">
         <v>96</v>
       </c>
@@ -4803,10 +5019,18 @@
       <c r="I36" s="7">
         <v>83</v>
       </c>
-      <c r="J36" s="8"/>
-      <c r="K36" s="8"/>
-      <c r="L36" s="8"/>
-      <c r="M36" s="8"/>
+      <c r="J36" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K36" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L36" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M36" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N36" s="5" t="s">
         <v>98</v>
       </c>
@@ -4839,10 +5063,18 @@
       <c r="I37" s="7">
         <v>10</v>
       </c>
-      <c r="J37" s="8"/>
-      <c r="K37" s="8"/>
-      <c r="L37" s="8"/>
-      <c r="M37" s="8"/>
+      <c r="J37" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K37" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L37" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M37" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N37" s="5" t="s">
         <v>100</v>
       </c>
@@ -4919,10 +5151,18 @@
       <c r="I39" s="7">
         <v>15</v>
       </c>
-      <c r="J39" s="8"/>
-      <c r="K39" s="8"/>
-      <c r="L39" s="8"/>
-      <c r="M39" s="8"/>
+      <c r="J39" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K39" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L39" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M39" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N39" s="5" t="s">
         <v>106</v>
       </c>
@@ -4999,10 +5239,18 @@
       <c r="I41" s="7">
         <v>56</v>
       </c>
-      <c r="J41" s="8"/>
-      <c r="K41" s="8"/>
-      <c r="L41" s="8"/>
-      <c r="M41" s="8"/>
+      <c r="J41" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K41" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L41" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M41" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N41" s="5" t="s">
         <v>110</v>
       </c>
@@ -5035,10 +5283,18 @@
       <c r="I42" s="7">
         <v>27</v>
       </c>
-      <c r="J42" s="8"/>
-      <c r="K42" s="8"/>
-      <c r="L42" s="8"/>
-      <c r="M42" s="8"/>
+      <c r="J42" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K42" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L42" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M42" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N42" s="5" t="s">
         <v>112</v>
       </c>
@@ -5071,10 +5327,18 @@
       <c r="I43" s="7">
         <v>40</v>
       </c>
-      <c r="J43" s="8"/>
-      <c r="K43" s="8"/>
-      <c r="L43" s="8"/>
-      <c r="M43" s="8"/>
+      <c r="J43" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K43" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L43" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M43" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N43" s="5" t="s">
         <v>114</v>
       </c>
@@ -5107,10 +5371,18 @@
       <c r="I44" s="7">
         <v>47</v>
       </c>
-      <c r="J44" s="8"/>
-      <c r="K44" s="8"/>
-      <c r="L44" s="8"/>
-      <c r="M44" s="8"/>
+      <c r="J44" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K44" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L44" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M44" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N44" s="5" t="s">
         <v>117</v>
       </c>
@@ -5231,10 +5503,18 @@
       <c r="I47" s="7">
         <v>15</v>
       </c>
-      <c r="J47" s="8"/>
-      <c r="K47" s="8"/>
-      <c r="L47" s="8"/>
-      <c r="M47" s="8"/>
+      <c r="J47" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K47" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L47" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M47" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N47" s="5" t="s">
         <v>123</v>
       </c>
@@ -5267,10 +5547,18 @@
       <c r="I48" s="7">
         <v>16</v>
       </c>
-      <c r="J48" s="8"/>
-      <c r="K48" s="8"/>
-      <c r="L48" s="8"/>
-      <c r="M48" s="8"/>
+      <c r="J48" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K48" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L48" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M48" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N48" s="5" t="s">
         <v>126</v>
       </c>
@@ -5303,10 +5591,18 @@
       <c r="I49" s="7">
         <v>13</v>
       </c>
-      <c r="J49" s="8"/>
-      <c r="K49" s="8"/>
-      <c r="L49" s="8"/>
-      <c r="M49" s="8"/>
+      <c r="J49" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K49" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L49" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M49" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N49" s="5" t="s">
         <v>128</v>
       </c>
@@ -5383,10 +5679,18 @@
       <c r="I51" s="7">
         <v>49</v>
       </c>
-      <c r="J51" s="8"/>
-      <c r="K51" s="8"/>
-      <c r="L51" s="8"/>
-      <c r="M51" s="8"/>
+      <c r="J51" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K51" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L51" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M51" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N51" s="5" t="s">
         <v>134</v>
       </c>
@@ -5463,10 +5767,18 @@
       <c r="I53" s="7">
         <v>21</v>
       </c>
-      <c r="J53" s="8"/>
-      <c r="K53" s="8"/>
-      <c r="L53" s="8"/>
-      <c r="M53" s="8"/>
+      <c r="J53" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K53" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L53" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M53" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N53" s="5" t="s">
         <v>139</v>
       </c>
@@ -5499,10 +5811,18 @@
       <c r="I54" s="7">
         <v>18</v>
       </c>
-      <c r="J54" s="8"/>
-      <c r="K54" s="8"/>
-      <c r="L54" s="8"/>
-      <c r="M54" s="8"/>
+      <c r="J54" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K54" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L54" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M54" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N54" s="5" t="s">
         <v>142</v>
       </c>
@@ -5535,10 +5855,18 @@
       <c r="I55" s="7">
         <v>17</v>
       </c>
-      <c r="J55" s="8"/>
-      <c r="K55" s="8"/>
-      <c r="L55" s="8"/>
-      <c r="M55" s="8"/>
+      <c r="J55" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K55" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L55" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M55" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N55" s="5" t="s">
         <v>144</v>
       </c>
@@ -5571,10 +5899,18 @@
       <c r="I56" s="7">
         <v>31</v>
       </c>
-      <c r="J56" s="8"/>
-      <c r="K56" s="8"/>
-      <c r="L56" s="8"/>
-      <c r="M56" s="8"/>
+      <c r="J56" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K56" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L56" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M56" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N56" s="5" t="s">
         <v>146</v>
       </c>
@@ -5607,10 +5943,18 @@
       <c r="I57" s="7">
         <v>35</v>
       </c>
-      <c r="J57" s="8"/>
-      <c r="K57" s="8"/>
-      <c r="L57" s="8"/>
-      <c r="M57" s="8"/>
+      <c r="J57" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K57" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L57" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M57" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N57" s="5" t="s">
         <v>148</v>
       </c>
@@ -5643,10 +5987,18 @@
       <c r="I58" s="7">
         <v>21</v>
       </c>
-      <c r="J58" s="8"/>
-      <c r="K58" s="8"/>
-      <c r="L58" s="8"/>
-      <c r="M58" s="8"/>
+      <c r="J58" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K58" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L58" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M58" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N58" s="5" t="s">
         <v>150</v>
       </c>
@@ -5855,10 +6207,18 @@
       <c r="I63" s="7">
         <v>18</v>
       </c>
-      <c r="J63" s="8"/>
-      <c r="K63" s="8"/>
-      <c r="L63" s="8"/>
-      <c r="M63" s="8"/>
+      <c r="J63" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K63" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L63" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M63" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N63" s="5" t="s">
         <v>163</v>
       </c>
@@ -5935,10 +6295,18 @@
       <c r="I65" s="7">
         <v>146</v>
       </c>
-      <c r="J65" s="8"/>
-      <c r="K65" s="8"/>
-      <c r="L65" s="8"/>
-      <c r="M65" s="8"/>
+      <c r="J65" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K65" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L65" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M65" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N65" s="5" t="s">
         <v>167</v>
       </c>
@@ -5971,10 +6339,18 @@
       <c r="I66" s="7">
         <v>31</v>
       </c>
-      <c r="J66" s="8"/>
-      <c r="K66" s="8"/>
-      <c r="L66" s="8"/>
-      <c r="M66" s="8"/>
+      <c r="J66" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K66" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L66" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M66" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N66" s="5" t="s">
         <v>169</v>
       </c>
@@ -6007,10 +6383,18 @@
       <c r="I67" s="7">
         <v>47</v>
       </c>
-      <c r="J67" s="8"/>
-      <c r="K67" s="8"/>
-      <c r="L67" s="8"/>
-      <c r="M67" s="8"/>
+      <c r="J67" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K67" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L67" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M67" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N67" s="5" t="s">
         <v>172</v>
       </c>
@@ -6043,10 +6427,18 @@
       <c r="I68" s="7">
         <v>18</v>
       </c>
-      <c r="J68" s="8"/>
-      <c r="K68" s="8"/>
-      <c r="L68" s="8"/>
-      <c r="M68" s="8"/>
+      <c r="J68" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K68" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L68" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M68" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N68" s="5" t="s">
         <v>175</v>
       </c>
@@ -6079,10 +6471,18 @@
       <c r="I69" s="7">
         <v>13</v>
       </c>
-      <c r="J69" s="8"/>
-      <c r="K69" s="8"/>
-      <c r="L69" s="8"/>
-      <c r="M69" s="8"/>
+      <c r="J69" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K69" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L69" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M69" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N69" s="5" t="s">
         <v>178</v>
       </c>
@@ -6115,10 +6515,18 @@
       <c r="I70" s="7">
         <v>11</v>
       </c>
-      <c r="J70" s="8"/>
-      <c r="K70" s="8"/>
-      <c r="L70" s="8"/>
-      <c r="M70" s="8"/>
+      <c r="J70" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K70" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L70" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M70" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N70" s="5" t="s">
         <v>180</v>
       </c>
@@ -6503,10 +6911,18 @@
       <c r="I79" s="7">
         <v>52</v>
       </c>
-      <c r="J79" s="8"/>
-      <c r="K79" s="8"/>
-      <c r="L79" s="8"/>
-      <c r="M79" s="8"/>
+      <c r="J79" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K79" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L79" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M79" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N79" s="5" t="s">
         <v>203</v>
       </c>
@@ -6539,10 +6955,18 @@
       <c r="I80" s="7">
         <v>39</v>
       </c>
-      <c r="J80" s="8"/>
-      <c r="K80" s="8"/>
-      <c r="L80" s="8"/>
-      <c r="M80" s="8"/>
+      <c r="J80" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K80" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L80" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M80" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N80" s="5" t="s">
         <v>206</v>
       </c>
@@ -6575,10 +6999,18 @@
       <c r="I81" s="7">
         <v>19</v>
       </c>
-      <c r="J81" s="8"/>
-      <c r="K81" s="8"/>
-      <c r="L81" s="8"/>
-      <c r="M81" s="8"/>
+      <c r="J81" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K81" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L81" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M81" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N81" s="5" t="s">
         <v>209</v>
       </c>
@@ -6611,10 +7043,18 @@
       <c r="I82" s="7">
         <v>20</v>
       </c>
-      <c r="J82" s="8"/>
-      <c r="K82" s="8"/>
-      <c r="L82" s="8"/>
-      <c r="M82" s="8"/>
+      <c r="J82" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K82" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L82" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M82" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N82" s="5" t="s">
         <v>211</v>
       </c>
@@ -6647,10 +7087,18 @@
       <c r="I83" s="7">
         <v>25</v>
       </c>
-      <c r="J83" s="8"/>
-      <c r="K83" s="8"/>
-      <c r="L83" s="8"/>
-      <c r="M83" s="8"/>
+      <c r="J83" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K83" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L83" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M83" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N83" s="5" t="s">
         <v>213</v>
       </c>
@@ -6727,10 +7175,18 @@
       <c r="I85" s="7">
         <v>40</v>
       </c>
-      <c r="J85" s="8"/>
-      <c r="K85" s="8"/>
-      <c r="L85" s="8"/>
-      <c r="M85" s="8"/>
+      <c r="J85" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K85" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L85" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M85" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N85" s="5" t="s">
         <v>218</v>
       </c>
@@ -6895,10 +7351,18 @@
       <c r="I89" s="7">
         <v>35</v>
       </c>
-      <c r="J89" s="8"/>
-      <c r="K89" s="8"/>
-      <c r="L89" s="8"/>
-      <c r="M89" s="8"/>
+      <c r="J89" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K89" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L89" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M89" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N89" s="5" t="s">
         <v>228</v>
       </c>
@@ -6931,10 +7395,18 @@
       <c r="I90" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J90" s="8"/>
-      <c r="K90" s="8"/>
-      <c r="L90" s="8"/>
-      <c r="M90" s="8"/>
+      <c r="J90" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K90" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L90" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M90" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N90" s="5" t="s">
         <v>230</v>
       </c>
@@ -6967,10 +7439,18 @@
       <c r="I91" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J91" s="8"/>
-      <c r="K91" s="8"/>
-      <c r="L91" s="8"/>
-      <c r="M91" s="8"/>
+      <c r="J91" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K91" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L91" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M91" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N91" s="5" t="s">
         <v>232</v>
       </c>
@@ -7091,10 +7571,18 @@
       <c r="I94" s="7">
         <v>12</v>
       </c>
-      <c r="J94" s="8"/>
-      <c r="K94" s="8"/>
-      <c r="L94" s="8"/>
-      <c r="M94" s="8"/>
+      <c r="J94" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K94" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L94" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M94" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N94" s="5" t="s">
         <v>240</v>
       </c>
@@ -7127,10 +7615,18 @@
       <c r="I95" s="7">
         <v>18</v>
       </c>
-      <c r="J95" s="8"/>
-      <c r="K95" s="8"/>
-      <c r="L95" s="8"/>
-      <c r="M95" s="8"/>
+      <c r="J95" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K95" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L95" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M95" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N95" s="5" t="s">
         <v>243</v>
       </c>
@@ -7251,10 +7747,18 @@
       <c r="I98" s="7">
         <v>32</v>
       </c>
-      <c r="J98" s="8"/>
-      <c r="K98" s="8"/>
-      <c r="L98" s="8"/>
-      <c r="M98" s="8"/>
+      <c r="J98" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K98" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L98" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M98" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N98" s="5" t="s">
         <v>249</v>
       </c>
@@ -7287,10 +7791,18 @@
       <c r="I99" s="7">
         <v>572</v>
       </c>
-      <c r="J99" s="8"/>
-      <c r="K99" s="8"/>
-      <c r="L99" s="8"/>
-      <c r="M99" s="8"/>
+      <c r="J99" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K99" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L99" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M99" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N99" s="5" t="s">
         <v>251</v>
       </c>
@@ -7323,10 +7835,18 @@
       <c r="I100" s="7">
         <v>84</v>
       </c>
-      <c r="J100" s="8"/>
-      <c r="K100" s="8"/>
-      <c r="L100" s="8"/>
-      <c r="M100" s="8"/>
+      <c r="J100" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K100" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L100" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M100" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N100" s="5" t="s">
         <v>253</v>
       </c>
@@ -7359,10 +7879,18 @@
       <c r="I101" s="7">
         <v>34</v>
       </c>
-      <c r="J101" s="8"/>
-      <c r="K101" s="8"/>
-      <c r="L101" s="8"/>
-      <c r="M101" s="8"/>
+      <c r="J101" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K101" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L101" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M101" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N101" s="5" t="s">
         <v>255</v>
       </c>
@@ -7395,10 +7923,18 @@
       <c r="I102" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J102" s="8"/>
-      <c r="K102" s="8"/>
-      <c r="L102" s="8"/>
-      <c r="M102" s="8"/>
+      <c r="J102" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K102" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L102" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M102" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N102" s="5" t="s">
         <v>257</v>
       </c>
@@ -7431,10 +7967,18 @@
       <c r="I103" s="7">
         <v>113</v>
       </c>
-      <c r="J103" s="8"/>
-      <c r="K103" s="8"/>
-      <c r="L103" s="8"/>
-      <c r="M103" s="8"/>
+      <c r="J103" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K103" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L103" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M103" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N103" s="5" t="s">
         <v>259</v>
       </c>
@@ -7467,10 +8011,18 @@
       <c r="I104" s="7">
         <v>879</v>
       </c>
-      <c r="J104" s="8"/>
-      <c r="K104" s="8"/>
-      <c r="L104" s="8"/>
-      <c r="M104" s="8"/>
+      <c r="J104" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K104" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L104" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M104" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N104" s="5" t="s">
         <v>261</v>
       </c>
@@ -7547,10 +8099,18 @@
       <c r="I106" s="7">
         <v>228</v>
       </c>
-      <c r="J106" s="7"/>
-      <c r="K106" s="9"/>
-      <c r="L106" s="9"/>
-      <c r="M106" s="9"/>
+      <c r="J106" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K106" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="L106" s="9" t="s">
+        <v>13</v>
+      </c>
+      <c r="M106" s="9" t="s">
+        <v>13</v>
+      </c>
       <c r="N106" s="5" t="s">
         <v>265</v>
       </c>
@@ -7583,10 +8143,18 @@
       <c r="I107" s="7">
         <v>91</v>
       </c>
-      <c r="J107" s="8"/>
-      <c r="K107" s="8"/>
-      <c r="L107" s="8"/>
-      <c r="M107" s="8"/>
+      <c r="J107" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K107" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L107" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M107" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N107" s="5" t="s">
         <v>267</v>
       </c>
@@ -7619,10 +8187,18 @@
       <c r="I108" s="7">
         <v>31</v>
       </c>
-      <c r="J108" s="8"/>
-      <c r="K108" s="8"/>
-      <c r="L108" s="8"/>
-      <c r="M108" s="8"/>
+      <c r="J108" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K108" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L108" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M108" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N108" s="5" t="s">
         <v>269</v>
       </c>
@@ -7655,10 +8231,18 @@
       <c r="I109" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J109" s="8"/>
-      <c r="K109" s="8"/>
-      <c r="L109" s="8"/>
-      <c r="M109" s="8"/>
+      <c r="J109" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K109" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L109" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M109" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N109" s="5" t="s">
         <v>271</v>
       </c>
@@ -7691,10 +8275,18 @@
       <c r="I110" s="7">
         <v>21</v>
       </c>
-      <c r="J110" s="8"/>
-      <c r="K110" s="8"/>
-      <c r="L110" s="8"/>
-      <c r="M110" s="8"/>
+      <c r="J110" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K110" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L110" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M110" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N110" s="5" t="s">
         <v>273</v>
       </c>
@@ -7727,10 +8319,18 @@
       <c r="I111" s="7">
         <v>52</v>
       </c>
-      <c r="J111" s="8"/>
-      <c r="K111" s="8"/>
-      <c r="L111" s="8"/>
-      <c r="M111" s="8"/>
+      <c r="J111" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K111" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L111" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M111" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N111" s="5" t="s">
         <v>275</v>
       </c>
@@ -7763,10 +8363,18 @@
       <c r="I112" s="7">
         <v>101</v>
       </c>
-      <c r="J112" s="8"/>
-      <c r="K112" s="8"/>
-      <c r="L112" s="8"/>
-      <c r="M112" s="8"/>
+      <c r="J112" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K112" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L112" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M112" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N112" s="5" t="s">
         <v>278</v>
       </c>
@@ -7799,10 +8407,18 @@
       <c r="I113" s="7">
         <v>96</v>
       </c>
-      <c r="J113" s="8"/>
-      <c r="K113" s="8"/>
-      <c r="L113" s="8"/>
-      <c r="M113" s="8"/>
+      <c r="J113" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K113" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L113" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M113" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N113" s="5" t="s">
         <v>280</v>
       </c>
@@ -7835,10 +8451,18 @@
       <c r="I114" s="7">
         <v>26</v>
       </c>
-      <c r="J114" s="8"/>
-      <c r="K114" s="8"/>
-      <c r="L114" s="8"/>
-      <c r="M114" s="8"/>
+      <c r="J114" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K114" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L114" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M114" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N114" s="5" t="s">
         <v>283</v>
       </c>
@@ -7871,10 +8495,18 @@
       <c r="I115" s="7">
         <v>15</v>
       </c>
-      <c r="J115" s="8"/>
-      <c r="K115" s="8"/>
-      <c r="L115" s="8"/>
-      <c r="M115" s="8"/>
+      <c r="J115" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K115" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L115" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M115" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N115" s="5" t="s">
         <v>285</v>
       </c>
@@ -7951,10 +8583,18 @@
       <c r="I117" s="7">
         <v>35</v>
       </c>
-      <c r="J117" s="8"/>
-      <c r="K117" s="8"/>
-      <c r="L117" s="8"/>
-      <c r="M117" s="8"/>
+      <c r="J117" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K117" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L117" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M117" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N117" s="5" t="s">
         <v>289</v>
       </c>
@@ -7987,10 +8627,18 @@
       <c r="I118" s="7">
         <v>13</v>
       </c>
-      <c r="J118" s="8"/>
-      <c r="K118" s="8"/>
-      <c r="L118" s="8"/>
-      <c r="M118" s="8"/>
+      <c r="J118" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K118" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L118" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M118" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N118" s="5" t="s">
         <v>291</v>
       </c>
@@ -8023,10 +8671,18 @@
       <c r="I119" s="7">
         <v>34</v>
       </c>
-      <c r="J119" s="8"/>
-      <c r="K119" s="8"/>
-      <c r="L119" s="8"/>
-      <c r="M119" s="8"/>
+      <c r="J119" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K119" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L119" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M119" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N119" s="5" t="s">
         <v>293</v>
       </c>
@@ -8059,10 +8715,18 @@
       <c r="I120" s="7">
         <v>15</v>
       </c>
-      <c r="J120" s="8"/>
-      <c r="K120" s="8"/>
-      <c r="L120" s="8"/>
-      <c r="M120" s="8"/>
+      <c r="J120" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K120" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L120" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M120" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N120" s="5" t="s">
         <v>295</v>
       </c>
@@ -8095,10 +8759,18 @@
       <c r="I121" s="7">
         <v>68</v>
       </c>
-      <c r="J121" s="8"/>
-      <c r="K121" s="8"/>
-      <c r="L121" s="8"/>
-      <c r="M121" s="8"/>
+      <c r="J121" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K121" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L121" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M121" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N121" s="5" t="s">
         <v>297</v>
       </c>
@@ -8131,10 +8803,18 @@
       <c r="I122" s="7">
         <v>47</v>
       </c>
-      <c r="J122" s="8"/>
-      <c r="K122" s="8"/>
-      <c r="L122" s="8"/>
-      <c r="M122" s="8"/>
+      <c r="J122" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K122" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L122" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M122" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N122" s="5" t="s">
         <v>300</v>
       </c>
@@ -8167,10 +8847,18 @@
       <c r="I123" s="7">
         <v>19</v>
       </c>
-      <c r="J123" s="8"/>
-      <c r="K123" s="8"/>
-      <c r="L123" s="8"/>
-      <c r="M123" s="8"/>
+      <c r="J123" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K123" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L123" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M123" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N123" s="5" t="s">
         <v>303</v>
       </c>
@@ -8203,10 +8891,18 @@
       <c r="I124" s="7">
         <v>20</v>
       </c>
-      <c r="J124" s="8"/>
-      <c r="K124" s="8"/>
-      <c r="L124" s="8"/>
-      <c r="M124" s="8"/>
+      <c r="J124" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K124" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L124" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M124" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N124" s="5" t="s">
         <v>304</v>
       </c>
@@ -8239,10 +8935,18 @@
       <c r="I125" s="7">
         <v>660</v>
       </c>
-      <c r="J125" s="8"/>
-      <c r="K125" s="8"/>
-      <c r="L125" s="8"/>
-      <c r="M125" s="8"/>
+      <c r="J125" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K125" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L125" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M125" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N125" s="5" t="s">
         <v>306</v>
       </c>
@@ -8275,10 +8979,18 @@
       <c r="I126" s="7">
         <v>70</v>
       </c>
-      <c r="J126" s="8"/>
-      <c r="K126" s="8"/>
-      <c r="L126" s="8"/>
-      <c r="M126" s="8"/>
+      <c r="J126" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K126" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L126" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M126" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N126" s="5" t="s">
         <v>308</v>
       </c>
@@ -8311,10 +9023,18 @@
       <c r="I127" s="7">
         <v>297</v>
       </c>
-      <c r="J127" s="8"/>
-      <c r="K127" s="8"/>
-      <c r="L127" s="8"/>
-      <c r="M127" s="8"/>
+      <c r="J127" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K127" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L127" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M127" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N127" s="5" t="s">
         <v>310</v>
       </c>
@@ -8347,10 +9067,18 @@
       <c r="I128" s="7">
         <v>92</v>
       </c>
-      <c r="J128" s="8"/>
-      <c r="K128" s="8"/>
-      <c r="L128" s="8"/>
-      <c r="M128" s="8"/>
+      <c r="J128" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K128" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L128" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M128" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N128" s="5" t="s">
         <v>312</v>
       </c>
@@ -8383,10 +9111,18 @@
       <c r="I129" s="7">
         <v>31</v>
       </c>
-      <c r="J129" s="8"/>
-      <c r="K129" s="8"/>
-      <c r="L129" s="8"/>
-      <c r="M129" s="8"/>
+      <c r="J129" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K129" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L129" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M129" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N129" s="5" t="s">
         <v>314</v>
       </c>
@@ -8463,10 +9199,18 @@
       <c r="I131" s="7">
         <v>78</v>
       </c>
-      <c r="J131" s="8"/>
-      <c r="K131" s="8"/>
-      <c r="L131" s="8"/>
-      <c r="M131" s="8"/>
+      <c r="J131" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K131" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L131" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M131" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N131" s="5" t="s">
         <v>318</v>
       </c>
@@ -8499,10 +9243,18 @@
       <c r="I132" s="7">
         <v>52</v>
       </c>
-      <c r="J132" s="8"/>
-      <c r="K132" s="8"/>
-      <c r="L132" s="8"/>
-      <c r="M132" s="8"/>
+      <c r="J132" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K132" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L132" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M132" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N132" s="5" t="s">
         <v>320</v>
       </c>
@@ -8579,10 +9331,18 @@
       <c r="I134" s="7">
         <v>30</v>
       </c>
-      <c r="J134" s="8"/>
-      <c r="K134" s="8"/>
-      <c r="L134" s="8"/>
-      <c r="M134" s="8"/>
+      <c r="J134" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K134" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L134" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M134" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N134" s="5" t="s">
         <v>325</v>
       </c>
@@ -8615,10 +9375,18 @@
       <c r="I135" s="7">
         <v>48</v>
       </c>
-      <c r="J135" s="8"/>
-      <c r="K135" s="8"/>
-      <c r="L135" s="8"/>
-      <c r="M135" s="8"/>
+      <c r="J135" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K135" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L135" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M135" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N135" s="5" t="s">
         <v>327</v>
       </c>
@@ -8651,10 +9419,18 @@
       <c r="I136" s="7">
         <v>24</v>
       </c>
-      <c r="J136" s="8"/>
-      <c r="K136" s="8"/>
-      <c r="L136" s="8"/>
-      <c r="M136" s="8"/>
+      <c r="J136" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K136" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L136" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M136" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N136" s="5" t="s">
         <v>330</v>
       </c>
@@ -8731,10 +9507,18 @@
       <c r="I138" s="7">
         <v>36</v>
       </c>
-      <c r="J138" s="8"/>
-      <c r="K138" s="8"/>
-      <c r="L138" s="8"/>
-      <c r="M138" s="8"/>
+      <c r="J138" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K138" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L138" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M138" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N138" s="5" t="s">
         <v>334</v>
       </c>
@@ -8767,10 +9551,18 @@
       <c r="I139" s="7">
         <v>31</v>
       </c>
-      <c r="J139" s="8"/>
-      <c r="K139" s="8"/>
-      <c r="L139" s="8"/>
-      <c r="M139" s="8"/>
+      <c r="J139" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K139" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L139" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M139" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N139" s="5" t="s">
         <v>336</v>
       </c>
@@ -8803,10 +9595,18 @@
       <c r="I140" s="7">
         <v>44</v>
       </c>
-      <c r="J140" s="8"/>
-      <c r="K140" s="8"/>
-      <c r="L140" s="8"/>
-      <c r="M140" s="8"/>
+      <c r="J140" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K140" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L140" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M140" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N140" s="5" t="s">
         <v>339</v>
       </c>
@@ -9015,10 +9815,18 @@
       <c r="I145" s="7">
         <v>27</v>
       </c>
-      <c r="J145" s="8"/>
-      <c r="K145" s="8"/>
-      <c r="L145" s="8"/>
-      <c r="M145" s="8"/>
+      <c r="J145" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K145" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L145" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M145" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N145" s="5" t="s">
         <v>349</v>
       </c>
@@ -9051,10 +9859,18 @@
       <c r="I146" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J146" s="8"/>
-      <c r="K146" s="8"/>
-      <c r="L146" s="8"/>
-      <c r="M146" s="8"/>
+      <c r="J146" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K146" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L146" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M146" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N146" s="5" t="s">
         <v>352</v>
       </c>
@@ -9175,10 +9991,18 @@
       <c r="I149" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J149" s="8"/>
-      <c r="K149" s="8"/>
-      <c r="L149" s="8"/>
-      <c r="M149" s="8"/>
+      <c r="J149" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K149" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L149" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M149" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N149" s="5" t="s">
         <v>352</v>
       </c>
@@ -9211,10 +10035,18 @@
       <c r="I150" s="7">
         <v>57</v>
       </c>
-      <c r="J150" s="8"/>
-      <c r="K150" s="8"/>
-      <c r="L150" s="8"/>
-      <c r="M150" s="8"/>
+      <c r="J150" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K150" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L150" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M150" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N150" s="5" t="s">
         <v>359</v>
       </c>
@@ -9247,10 +10079,18 @@
       <c r="I151" s="7">
         <v>165</v>
       </c>
-      <c r="J151" s="8"/>
-      <c r="K151" s="8"/>
-      <c r="L151" s="8"/>
-      <c r="M151" s="8"/>
+      <c r="J151" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K151" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L151" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M151" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N151" s="5" t="s">
         <v>362</v>
       </c>
@@ -9415,10 +10255,18 @@
       <c r="I155" s="7">
         <v>33</v>
       </c>
-      <c r="J155" s="8"/>
-      <c r="K155" s="8"/>
-      <c r="L155" s="8"/>
-      <c r="M155" s="8"/>
+      <c r="J155" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K155" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L155" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M155" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N155" s="5" t="s">
         <v>373</v>
       </c>
@@ -9451,10 +10299,18 @@
       <c r="I156" s="7">
         <v>25</v>
       </c>
-      <c r="J156" s="8"/>
-      <c r="K156" s="8"/>
-      <c r="L156" s="8"/>
-      <c r="M156" s="8"/>
+      <c r="J156" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K156" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L156" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M156" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N156" s="5" t="s">
         <v>376</v>
       </c>
@@ -9531,10 +10387,18 @@
       <c r="I158" s="7">
         <v>65</v>
       </c>
-      <c r="J158" s="8"/>
-      <c r="K158" s="8"/>
-      <c r="L158" s="8"/>
-      <c r="M158" s="8"/>
+      <c r="J158" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K158" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L158" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M158" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N158" s="5" t="s">
         <v>383</v>
       </c>
@@ -9567,10 +10431,18 @@
       <c r="I159" s="7">
         <v>44</v>
       </c>
-      <c r="J159" s="8"/>
-      <c r="K159" s="8"/>
-      <c r="L159" s="8"/>
-      <c r="M159" s="8"/>
+      <c r="J159" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K159" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L159" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M159" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N159" s="5" t="s">
         <v>386</v>
       </c>
@@ -9603,10 +10475,18 @@
       <c r="I160" s="7">
         <v>50</v>
       </c>
-      <c r="J160" s="8"/>
-      <c r="K160" s="8"/>
-      <c r="L160" s="8"/>
-      <c r="M160" s="8"/>
+      <c r="J160" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K160" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L160" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M160" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N160" s="5" t="s">
         <v>388</v>
       </c>
@@ -9683,10 +10563,18 @@
       <c r="I162" s="7">
         <v>31</v>
       </c>
-      <c r="J162" s="8"/>
-      <c r="K162" s="8"/>
-      <c r="L162" s="8"/>
-      <c r="M162" s="8"/>
+      <c r="J162" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K162" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L162" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M162" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N162" s="5" t="s">
         <v>393</v>
       </c>
@@ -9719,10 +10607,18 @@
       <c r="I163" s="7">
         <v>20</v>
       </c>
-      <c r="J163" s="8"/>
-      <c r="K163" s="8"/>
-      <c r="L163" s="8"/>
-      <c r="M163" s="8"/>
+      <c r="J163" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K163" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L163" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M163" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N163" s="5" t="s">
         <v>395</v>
       </c>
@@ -9755,10 +10651,18 @@
       <c r="I164" s="17">
         <v>861</v>
       </c>
-      <c r="J164" s="19"/>
-      <c r="K164" s="19"/>
-      <c r="L164" s="19"/>
-      <c r="M164" s="19"/>
+      <c r="J164" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="K164" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="L164" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="M164" s="19" t="s">
+        <v>13</v>
+      </c>
       <c r="N164" s="13" t="s">
         <v>397</v>
       </c>
@@ -9807,10 +10711,18 @@
       <c r="I166" s="17">
         <v>477</v>
       </c>
-      <c r="J166" s="19"/>
-      <c r="K166" s="19"/>
-      <c r="L166" s="19"/>
-      <c r="M166" s="19"/>
+      <c r="J166" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="K166" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="L166" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="M166" s="19" t="s">
+        <v>13</v>
+      </c>
       <c r="N166" s="13" t="s">
         <v>400</v>
       </c>
@@ -9859,10 +10771,18 @@
       <c r="I168" s="7">
         <v>115</v>
       </c>
-      <c r="J168" s="8"/>
-      <c r="K168" s="8"/>
-      <c r="L168" s="8"/>
-      <c r="M168" s="8"/>
+      <c r="J168" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K168" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L168" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M168" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N168" s="5" t="s">
         <v>403</v>
       </c>
@@ -9895,10 +10815,18 @@
       <c r="I169" s="7">
         <v>24</v>
       </c>
-      <c r="J169" s="8"/>
-      <c r="K169" s="8"/>
-      <c r="L169" s="8"/>
-      <c r="M169" s="8"/>
+      <c r="J169" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K169" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L169" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M169" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N169" s="5" t="s">
         <v>406</v>
       </c>
@@ -9931,10 +10859,18 @@
       <c r="I170" s="7">
         <v>40</v>
       </c>
-      <c r="J170" s="8"/>
-      <c r="K170" s="8"/>
-      <c r="L170" s="8"/>
-      <c r="M170" s="8"/>
+      <c r="J170" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K170" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L170" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M170" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N170" s="5" t="s">
         <v>409</v>
       </c>
@@ -10055,10 +10991,18 @@
       <c r="I173" s="7">
         <v>33</v>
       </c>
-      <c r="J173" s="8"/>
-      <c r="K173" s="8"/>
-      <c r="L173" s="8"/>
-      <c r="M173" s="8"/>
+      <c r="J173" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K173" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L173" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M173" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N173" s="5" t="s">
         <v>419</v>
       </c>
@@ -10091,10 +11035,18 @@
       <c r="I174" s="7">
         <v>199</v>
       </c>
-      <c r="J174" s="8"/>
-      <c r="K174" s="8"/>
-      <c r="L174" s="8"/>
-      <c r="M174" s="8"/>
+      <c r="J174" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K174" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L174" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M174" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N174" s="5" t="s">
         <v>422</v>
       </c>
@@ -10127,10 +11079,18 @@
       <c r="I175" s="7">
         <v>120</v>
       </c>
-      <c r="J175" s="8"/>
-      <c r="K175" s="8"/>
-      <c r="L175" s="8"/>
-      <c r="M175" s="8"/>
+      <c r="J175" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K175" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L175" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M175" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N175" s="5" t="s">
         <v>425</v>
       </c>
@@ -10163,10 +11123,18 @@
       <c r="I176" s="7">
         <v>132</v>
       </c>
-      <c r="J176" s="8"/>
-      <c r="K176" s="8"/>
-      <c r="L176" s="8"/>
-      <c r="M176" s="8"/>
+      <c r="J176" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K176" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L176" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M176" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N176" s="5" t="s">
         <v>428</v>
       </c>
@@ -10199,10 +11167,18 @@
       <c r="I177" s="7">
         <v>160</v>
       </c>
-      <c r="J177" s="8"/>
-      <c r="K177" s="8"/>
-      <c r="L177" s="8"/>
-      <c r="M177" s="8"/>
+      <c r="J177" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K177" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L177" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M177" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N177" s="5" t="s">
         <v>431</v>
       </c>
@@ -10235,10 +11211,18 @@
       <c r="I178" s="7">
         <v>511</v>
       </c>
-      <c r="J178" s="8"/>
-      <c r="K178" s="8"/>
-      <c r="L178" s="8"/>
-      <c r="M178" s="8"/>
+      <c r="J178" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K178" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L178" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M178" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N178" s="5" t="s">
         <v>435</v>
       </c>
@@ -10271,10 +11255,18 @@
       <c r="I179" s="7">
         <v>75</v>
       </c>
-      <c r="J179" s="8"/>
-      <c r="K179" s="8"/>
-      <c r="L179" s="8"/>
-      <c r="M179" s="8"/>
+      <c r="J179" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K179" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L179" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M179" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N179" s="5" t="s">
         <v>438</v>
       </c>
@@ -10351,10 +11343,18 @@
       <c r="I181" s="7">
         <v>91</v>
       </c>
-      <c r="J181" s="8"/>
-      <c r="K181" s="8"/>
-      <c r="L181" s="8"/>
-      <c r="M181" s="8"/>
+      <c r="J181" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K181" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L181" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M181" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N181" s="5" t="s">
         <v>445</v>
       </c>
@@ -10387,10 +11387,18 @@
       <c r="I182" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J182" s="8"/>
-      <c r="K182" s="8"/>
-      <c r="L182" s="8"/>
-      <c r="M182" s="8"/>
+      <c r="J182" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K182" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L182" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M182" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N182" s="5" t="s">
         <v>448</v>
       </c>
@@ -10555,10 +11563,18 @@
       <c r="I186" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J186" s="8"/>
-      <c r="K186" s="8"/>
-      <c r="L186" s="8"/>
-      <c r="M186" s="8"/>
+      <c r="J186" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K186" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L186" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M186" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N186" s="5" t="s">
         <v>462</v>
       </c>
@@ -10723,10 +11739,18 @@
       <c r="I190" s="7">
         <v>25</v>
       </c>
-      <c r="J190" s="8"/>
-      <c r="K190" s="8"/>
-      <c r="L190" s="8"/>
-      <c r="M190" s="8"/>
+      <c r="J190" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K190" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L190" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M190" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N190" s="5" t="s">
         <v>479</v>
       </c>
@@ -10803,10 +11827,18 @@
       <c r="I192" s="7">
         <v>25</v>
       </c>
-      <c r="J192" s="8"/>
-      <c r="K192" s="8"/>
-      <c r="L192" s="8"/>
-      <c r="M192" s="8"/>
+      <c r="J192" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K192" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L192" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M192" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N192" s="5" t="s">
         <v>487</v>
       </c>
@@ -10927,10 +11959,18 @@
       <c r="I195" s="7">
         <v>149</v>
       </c>
-      <c r="J195" s="8"/>
-      <c r="K195" s="8"/>
-      <c r="L195" s="8"/>
-      <c r="M195" s="8"/>
+      <c r="J195" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K195" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L195" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M195" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N195" s="5" t="s">
         <v>498</v>
       </c>
@@ -11095,10 +12135,18 @@
       <c r="I199" s="7">
         <v>18</v>
       </c>
-      <c r="J199" s="8"/>
-      <c r="K199" s="8"/>
-      <c r="L199" s="8"/>
-      <c r="M199" s="8"/>
+      <c r="J199" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K199" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L199" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M199" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N199" s="5" t="s">
         <v>511</v>
       </c>
@@ -11131,10 +12179,18 @@
       <c r="I200" s="7">
         <v>93</v>
       </c>
-      <c r="J200" s="8"/>
-      <c r="K200" s="8"/>
-      <c r="L200" s="8"/>
-      <c r="M200" s="8"/>
+      <c r="J200" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K200" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L200" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M200" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N200" s="5" t="s">
         <v>514</v>
       </c>
@@ -11387,10 +12443,18 @@
       <c r="I206" s="7">
         <v>102</v>
       </c>
-      <c r="J206" s="8"/>
-      <c r="K206" s="8"/>
-      <c r="L206" s="8"/>
-      <c r="M206" s="8"/>
+      <c r="J206" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K206" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L206" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M206" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N206" s="5" t="s">
         <v>532</v>
       </c>
@@ -11555,10 +12619,18 @@
       <c r="I210" s="7">
         <v>9</v>
       </c>
-      <c r="J210" s="8"/>
-      <c r="K210" s="8"/>
-      <c r="L210" s="8"/>
-      <c r="M210" s="8"/>
+      <c r="J210" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K210" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L210" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M210" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N210" s="5" t="s">
         <v>545</v>
       </c>
@@ -11591,10 +12663,18 @@
       <c r="I211" s="7">
         <v>50</v>
       </c>
-      <c r="J211" s="8"/>
-      <c r="K211" s="8"/>
-      <c r="L211" s="8"/>
-      <c r="M211" s="8"/>
+      <c r="J211" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K211" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L211" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M211" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N211" s="5" t="s">
         <v>548</v>
       </c>
@@ -11627,10 +12707,18 @@
       <c r="I212" s="7">
         <v>19</v>
       </c>
-      <c r="J212" s="8"/>
-      <c r="K212" s="8"/>
-      <c r="L212" s="8"/>
-      <c r="M212" s="8"/>
+      <c r="J212" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K212" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L212" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M212" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N212" s="5" t="s">
         <v>552</v>
       </c>
@@ -11663,10 +12751,18 @@
       <c r="I213" s="7">
         <v>17</v>
       </c>
-      <c r="J213" s="8"/>
-      <c r="K213" s="8"/>
-      <c r="L213" s="8"/>
-      <c r="M213" s="8"/>
+      <c r="J213" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K213" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L213" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M213" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N213" s="5" t="s">
         <v>555</v>
       </c>
@@ -11699,10 +12795,18 @@
       <c r="I214" s="7">
         <v>31</v>
       </c>
-      <c r="J214" s="8"/>
-      <c r="K214" s="8"/>
-      <c r="L214" s="8"/>
-      <c r="M214" s="8"/>
+      <c r="J214" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K214" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L214" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M214" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N214" s="5" t="s">
         <v>558</v>
       </c>
@@ -11911,10 +13015,18 @@
       <c r="I219" s="7">
         <v>31</v>
       </c>
-      <c r="J219" s="8"/>
-      <c r="K219" s="8"/>
-      <c r="L219" s="8"/>
-      <c r="M219" s="8"/>
+      <c r="J219" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K219" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L219" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M219" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N219" s="5" t="s">
         <v>575</v>
       </c>
@@ -11947,10 +13059,18 @@
       <c r="I220" s="7">
         <v>23</v>
       </c>
-      <c r="J220" s="8"/>
-      <c r="K220" s="8"/>
-      <c r="L220" s="8"/>
-      <c r="M220" s="8"/>
+      <c r="J220" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K220" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L220" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M220" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N220" s="5" t="s">
         <v>578</v>
       </c>
@@ -11983,10 +13103,18 @@
       <c r="I221" s="7">
         <v>50</v>
       </c>
-      <c r="J221" s="8"/>
-      <c r="K221" s="8"/>
-      <c r="L221" s="8"/>
-      <c r="M221" s="8"/>
+      <c r="J221" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K221" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L221" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M221" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N221" s="5" t="s">
         <v>581</v>
       </c>
@@ -12019,10 +13147,18 @@
       <c r="I222" s="7">
         <v>51</v>
       </c>
-      <c r="J222" s="8"/>
-      <c r="K222" s="8"/>
-      <c r="L222" s="8"/>
-      <c r="M222" s="8"/>
+      <c r="J222" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K222" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L222" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M222" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N222" s="5" t="s">
         <v>584</v>
       </c>
@@ -12055,10 +13191,18 @@
       <c r="I223" s="7">
         <v>973</v>
       </c>
-      <c r="J223" s="8"/>
-      <c r="K223" s="8"/>
-      <c r="L223" s="8"/>
-      <c r="M223" s="8"/>
+      <c r="J223" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K223" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L223" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M223" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N223" s="5" t="s">
         <v>587</v>
       </c>
@@ -12135,10 +13279,18 @@
       <c r="I225" s="7">
         <v>51</v>
       </c>
-      <c r="J225" s="8"/>
-      <c r="K225" s="8"/>
-      <c r="L225" s="8"/>
-      <c r="M225" s="8"/>
+      <c r="J225" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K225" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L225" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M225" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N225" s="5" t="s">
         <v>594</v>
       </c>
@@ -12171,11 +13323,21 @@
       <c r="I226" s="17">
         <v>472</v>
       </c>
-      <c r="J226" s="19"/>
-      <c r="K226" s="19"/>
-      <c r="L226" s="19"/>
-      <c r="M226" s="19"/>
-      <c r="N226" s="10"/>
+      <c r="J226" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="K226" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="L226" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="M226" s="19" t="s">
+        <v>13</v>
+      </c>
+      <c r="N226" s="10" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="227" spans="1:14" ht="17" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A227" s="16"/>
@@ -12223,10 +13385,18 @@
       <c r="I228" s="7">
         <v>55</v>
       </c>
-      <c r="J228" s="8"/>
-      <c r="K228" s="8"/>
-      <c r="L228" s="8"/>
-      <c r="M228" s="8"/>
+      <c r="J228" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K228" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L228" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M228" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N228" s="5" t="s">
         <v>600</v>
       </c>
@@ -12259,10 +13429,18 @@
       <c r="I229" s="7">
         <v>53</v>
       </c>
-      <c r="J229" s="8"/>
-      <c r="K229" s="8"/>
-      <c r="L229" s="8"/>
-      <c r="M229" s="8"/>
+      <c r="J229" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K229" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L229" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M229" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N229" s="5" t="s">
         <v>603</v>
       </c>
@@ -12295,10 +13473,18 @@
       <c r="I230" s="7">
         <v>38</v>
       </c>
-      <c r="J230" s="8"/>
-      <c r="K230" s="8"/>
-      <c r="L230" s="8"/>
-      <c r="M230" s="8"/>
+      <c r="J230" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K230" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L230" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M230" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N230" s="5" t="s">
         <v>606</v>
       </c>
@@ -12331,10 +13517,18 @@
       <c r="I231" s="7">
         <v>329</v>
       </c>
-      <c r="J231" s="8"/>
-      <c r="K231" s="8"/>
-      <c r="L231" s="8"/>
-      <c r="M231" s="8"/>
+      <c r="J231" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K231" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L231" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M231" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N231" s="5" t="s">
         <v>609</v>
       </c>
@@ -12411,10 +13605,18 @@
       <c r="I233" s="7">
         <v>21</v>
       </c>
-      <c r="J233" s="8"/>
-      <c r="K233" s="8"/>
-      <c r="L233" s="8"/>
-      <c r="M233" s="8"/>
+      <c r="J233" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K233" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L233" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M233" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N233" s="5" t="s">
         <v>615</v>
       </c>
@@ -12447,10 +13649,18 @@
       <c r="I234" s="7">
         <v>11</v>
       </c>
-      <c r="J234" s="8"/>
-      <c r="K234" s="8"/>
-      <c r="L234" s="8"/>
-      <c r="M234" s="8"/>
+      <c r="J234" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K234" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L234" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M234" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N234" s="5" t="s">
         <v>618</v>
       </c>
@@ -12483,10 +13693,18 @@
       <c r="I235" s="7">
         <v>19</v>
       </c>
-      <c r="J235" s="8"/>
-      <c r="K235" s="8"/>
-      <c r="L235" s="8"/>
-      <c r="M235" s="8"/>
+      <c r="J235" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K235" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L235" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M235" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N235" s="5" t="s">
         <v>621</v>
       </c>
@@ -12519,10 +13737,18 @@
       <c r="I236" s="7">
         <v>74</v>
       </c>
-      <c r="J236" s="8"/>
-      <c r="K236" s="8"/>
-      <c r="L236" s="8"/>
-      <c r="M236" s="8"/>
+      <c r="J236" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K236" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L236" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M236" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N236" s="5" t="s">
         <v>624</v>
       </c>
@@ -12555,10 +13781,18 @@
       <c r="I237" s="7">
         <v>15</v>
       </c>
-      <c r="J237" s="8"/>
-      <c r="K237" s="8"/>
-      <c r="L237" s="8"/>
-      <c r="M237" s="8"/>
+      <c r="J237" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K237" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L237" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M237" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N237" s="5" t="s">
         <v>628</v>
       </c>
@@ -12591,10 +13825,18 @@
       <c r="I238" s="7">
         <v>13</v>
       </c>
-      <c r="J238" s="8"/>
-      <c r="K238" s="8"/>
-      <c r="L238" s="8"/>
-      <c r="M238" s="8"/>
+      <c r="J238" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K238" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L238" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M238" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N238" s="5" t="s">
         <v>628</v>
       </c>
@@ -12627,10 +13869,18 @@
       <c r="I239" s="7">
         <v>39</v>
       </c>
-      <c r="J239" s="8"/>
-      <c r="K239" s="8"/>
-      <c r="L239" s="8"/>
-      <c r="M239" s="8"/>
+      <c r="J239" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K239" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L239" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M239" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N239" s="5" t="s">
         <v>633</v>
       </c>
@@ -12707,10 +13957,18 @@
       <c r="I241" s="7">
         <v>67</v>
       </c>
-      <c r="J241" s="8"/>
-      <c r="K241" s="8"/>
-      <c r="L241" s="8"/>
-      <c r="M241" s="8"/>
+      <c r="J241" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K241" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L241" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M241" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N241" s="5" t="s">
         <v>639</v>
       </c>
@@ -12743,10 +14001,18 @@
       <c r="I242" s="7">
         <v>16</v>
       </c>
-      <c r="J242" s="8"/>
-      <c r="K242" s="8"/>
-      <c r="L242" s="8"/>
-      <c r="M242" s="8"/>
+      <c r="J242" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K242" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L242" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M242" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N242" s="5" t="s">
         <v>642</v>
       </c>
@@ -12779,10 +14045,18 @@
       <c r="I243" s="7">
         <v>20</v>
       </c>
-      <c r="J243" s="8"/>
-      <c r="K243" s="8"/>
-      <c r="L243" s="8"/>
-      <c r="M243" s="8"/>
+      <c r="J243" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K243" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L243" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M243" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N243" s="5" t="s">
         <v>645</v>
       </c>
@@ -12815,10 +14089,18 @@
       <c r="I244" s="7">
         <v>42</v>
       </c>
-      <c r="J244" s="8"/>
-      <c r="K244" s="8"/>
-      <c r="L244" s="8"/>
-      <c r="M244" s="8"/>
+      <c r="J244" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K244" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L244" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M244" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N244" s="5" t="s">
         <v>648</v>
       </c>
@@ -12851,10 +14133,18 @@
       <c r="I245" s="7">
         <v>109</v>
       </c>
-      <c r="J245" s="8"/>
-      <c r="K245" s="8"/>
-      <c r="L245" s="8"/>
-      <c r="M245" s="8"/>
+      <c r="J245" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K245" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L245" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M245" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N245" s="5" t="s">
         <v>651</v>
       </c>
@@ -12887,10 +14177,18 @@
       <c r="I246" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J246" s="8"/>
-      <c r="K246" s="8"/>
-      <c r="L246" s="8"/>
-      <c r="M246" s="8"/>
+      <c r="J246" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K246" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L246" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M246" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N246" s="5" t="s">
         <v>655</v>
       </c>
@@ -12923,10 +14221,18 @@
       <c r="I247" s="7">
         <v>7</v>
       </c>
-      <c r="J247" s="8"/>
-      <c r="K247" s="8"/>
-      <c r="L247" s="8"/>
-      <c r="M247" s="8"/>
+      <c r="J247" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K247" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L247" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M247" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N247" s="5" t="s">
         <v>658</v>
       </c>
@@ -12959,10 +14265,18 @@
       <c r="I248" s="7">
         <v>16</v>
       </c>
-      <c r="J248" s="8"/>
-      <c r="K248" s="8"/>
-      <c r="L248" s="8"/>
-      <c r="M248" s="8"/>
+      <c r="J248" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K248" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L248" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M248" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N248" s="5" t="s">
         <v>658</v>
       </c>
@@ -12995,10 +14309,18 @@
       <c r="I249" s="7">
         <v>53</v>
       </c>
-      <c r="J249" s="8"/>
-      <c r="K249" s="8"/>
-      <c r="L249" s="8"/>
-      <c r="M249" s="8"/>
+      <c r="J249" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K249" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L249" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M249" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N249" s="5" t="s">
         <v>664</v>
       </c>
@@ -13119,10 +14441,18 @@
       <c r="I252" s="7">
         <v>50</v>
       </c>
-      <c r="J252" s="8"/>
-      <c r="K252" s="8"/>
-      <c r="L252" s="8"/>
-      <c r="M252" s="8"/>
+      <c r="J252" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K252" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L252" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M252" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N252" s="5" t="s">
         <v>675</v>
       </c>
@@ -13287,10 +14617,18 @@
       <c r="I256" s="7">
         <v>407</v>
       </c>
-      <c r="J256" s="8"/>
-      <c r="K256" s="8"/>
-      <c r="L256" s="8"/>
-      <c r="M256" s="8"/>
+      <c r="J256" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K256" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L256" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M256" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N256" s="5" t="s">
         <v>688</v>
       </c>
@@ -13323,10 +14661,18 @@
       <c r="I257" s="7">
         <v>170</v>
       </c>
-      <c r="J257" s="8"/>
-      <c r="K257" s="8"/>
-      <c r="L257" s="8"/>
-      <c r="M257" s="8"/>
+      <c r="J257" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K257" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L257" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M257" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N257" s="5" t="s">
         <v>691</v>
       </c>
@@ -13359,10 +14705,18 @@
       <c r="I258" s="7">
         <v>29</v>
       </c>
-      <c r="J258" s="8"/>
-      <c r="K258" s="8"/>
-      <c r="L258" s="8"/>
-      <c r="M258" s="8"/>
+      <c r="J258" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K258" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L258" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M258" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N258" s="5" t="s">
         <v>694</v>
       </c>
@@ -13395,10 +14749,18 @@
       <c r="I259" s="7">
         <v>83</v>
       </c>
-      <c r="J259" s="8"/>
-      <c r="K259" s="8"/>
-      <c r="L259" s="8"/>
-      <c r="M259" s="8"/>
+      <c r="J259" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K259" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L259" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M259" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N259" s="5" t="s">
         <v>697</v>
       </c>
@@ -13431,10 +14793,18 @@
       <c r="I260" s="7">
         <v>87</v>
       </c>
-      <c r="J260" s="8"/>
-      <c r="K260" s="8"/>
-      <c r="L260" s="8"/>
-      <c r="M260" s="8"/>
+      <c r="J260" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K260" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L260" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M260" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N260" s="5" t="s">
         <v>697</v>
       </c>
@@ -13467,10 +14837,18 @@
       <c r="I261" s="7">
         <v>42</v>
       </c>
-      <c r="J261" s="8"/>
-      <c r="K261" s="8"/>
-      <c r="L261" s="8"/>
-      <c r="M261" s="8"/>
+      <c r="J261" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K261" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L261" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M261" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N261" s="5" t="s">
         <v>703</v>
       </c>
@@ -13503,10 +14881,18 @@
       <c r="I262" s="7">
         <v>63</v>
       </c>
-      <c r="J262" s="8"/>
-      <c r="K262" s="8"/>
-      <c r="L262" s="8"/>
-      <c r="M262" s="8"/>
+      <c r="J262" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K262" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L262" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M262" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N262" s="5" t="s">
         <v>707</v>
       </c>
@@ -13539,10 +14925,18 @@
       <c r="I263" s="7">
         <v>83</v>
       </c>
-      <c r="J263" s="8"/>
-      <c r="K263" s="8"/>
-      <c r="L263" s="8"/>
-      <c r="M263" s="8"/>
+      <c r="J263" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K263" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L263" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M263" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N263" s="5" t="s">
         <v>711</v>
       </c>
@@ -13575,10 +14969,18 @@
       <c r="I264" s="7">
         <v>98</v>
       </c>
-      <c r="J264" s="8"/>
-      <c r="K264" s="8"/>
-      <c r="L264" s="8"/>
-      <c r="M264" s="8"/>
+      <c r="J264" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K264" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L264" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M264" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N264" s="5" t="s">
         <v>714</v>
       </c>
@@ -13611,10 +15013,18 @@
       <c r="I265" s="7">
         <v>28</v>
       </c>
-      <c r="J265" s="8"/>
-      <c r="K265" s="8"/>
-      <c r="L265" s="8"/>
-      <c r="M265" s="8"/>
+      <c r="J265" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K265" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L265" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M265" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N265" s="5" t="s">
         <v>717</v>
       </c>
@@ -13647,10 +15057,18 @@
       <c r="I266" s="7">
         <v>34</v>
       </c>
-      <c r="J266" s="8"/>
-      <c r="K266" s="8"/>
-      <c r="L266" s="8"/>
-      <c r="M266" s="8"/>
+      <c r="J266" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K266" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L266" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M266" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N266" s="5" t="s">
         <v>720</v>
       </c>
@@ -13683,10 +15101,18 @@
       <c r="I267" s="7">
         <v>41</v>
       </c>
-      <c r="J267" s="8"/>
-      <c r="K267" s="8"/>
-      <c r="L267" s="8"/>
-      <c r="M267" s="8"/>
+      <c r="J267" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K267" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L267" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M267" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N267" s="5" t="s">
         <v>723</v>
       </c>
@@ -13719,10 +15145,18 @@
       <c r="I268" s="7">
         <v>49</v>
       </c>
-      <c r="J268" s="8"/>
-      <c r="K268" s="8"/>
-      <c r="L268" s="8"/>
-      <c r="M268" s="8"/>
+      <c r="J268" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K268" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L268" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M268" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N268" s="5" t="s">
         <v>727</v>
       </c>
@@ -13755,10 +15189,18 @@
       <c r="I269" s="7">
         <v>13</v>
       </c>
-      <c r="J269" s="8"/>
-      <c r="K269" s="8"/>
-      <c r="L269" s="8"/>
-      <c r="M269" s="8"/>
+      <c r="J269" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K269" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L269" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M269" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N269" s="5" t="s">
         <v>731</v>
       </c>
@@ -13791,10 +15233,18 @@
       <c r="I270" s="7">
         <v>18</v>
       </c>
-      <c r="J270" s="8"/>
-      <c r="K270" s="8"/>
-      <c r="L270" s="8"/>
-      <c r="M270" s="8"/>
+      <c r="J270" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K270" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L270" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M270" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N270" s="5" t="s">
         <v>734</v>
       </c>
@@ -13827,10 +15277,18 @@
       <c r="I271" s="7">
         <v>38</v>
       </c>
-      <c r="J271" s="8"/>
-      <c r="K271" s="8"/>
-      <c r="L271" s="8"/>
-      <c r="M271" s="8"/>
+      <c r="J271" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K271" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L271" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M271" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N271" s="5" t="s">
         <v>737</v>
       </c>
@@ -13863,10 +15321,18 @@
       <c r="I272" s="7">
         <v>21</v>
       </c>
-      <c r="J272" s="8"/>
-      <c r="K272" s="8"/>
-      <c r="L272" s="8"/>
-      <c r="M272" s="8"/>
+      <c r="J272" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K272" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L272" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M272" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N272" s="5" t="s">
         <v>740</v>
       </c>
@@ -13899,10 +15365,18 @@
       <c r="I273" s="7">
         <v>32</v>
       </c>
-      <c r="J273" s="8"/>
-      <c r="K273" s="8"/>
-      <c r="L273" s="8"/>
-      <c r="M273" s="8"/>
+      <c r="J273" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K273" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L273" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M273" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N273" s="5" t="s">
         <v>744</v>
       </c>
@@ -13935,10 +15409,18 @@
       <c r="I274" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="J274" s="8"/>
-      <c r="K274" s="8"/>
-      <c r="L274" s="8"/>
-      <c r="M274" s="8"/>
+      <c r="J274" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K274" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L274" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M274" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N274" s="5" t="s">
         <v>747</v>
       </c>
@@ -13971,10 +15453,18 @@
       <c r="I275" s="7">
         <v>16</v>
       </c>
-      <c r="J275" s="8"/>
-      <c r="K275" s="8"/>
-      <c r="L275" s="8"/>
-      <c r="M275" s="8"/>
+      <c r="J275" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K275" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L275" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M275" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N275" s="5" t="s">
         <v>750</v>
       </c>
@@ -14007,10 +15497,18 @@
       <c r="I276" s="7">
         <v>23</v>
       </c>
-      <c r="J276" s="8"/>
-      <c r="K276" s="8"/>
-      <c r="L276" s="8"/>
-      <c r="M276" s="8"/>
+      <c r="J276" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K276" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L276" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M276" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N276" s="5" t="s">
         <v>753</v>
       </c>
@@ -14043,10 +15541,18 @@
       <c r="I277" s="7">
         <v>52</v>
       </c>
-      <c r="J277" s="8"/>
-      <c r="K277" s="8"/>
-      <c r="L277" s="8"/>
-      <c r="M277" s="8"/>
+      <c r="J277" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K277" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L277" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M277" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N277" s="5" t="s">
         <v>756</v>
       </c>
@@ -14079,10 +15585,18 @@
       <c r="I278" s="7">
         <v>17</v>
       </c>
-      <c r="J278" s="8"/>
-      <c r="K278" s="8"/>
-      <c r="L278" s="8"/>
-      <c r="M278" s="8"/>
+      <c r="J278" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K278" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L278" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M278" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N278" s="5" t="s">
         <v>759</v>
       </c>
@@ -14115,10 +15629,18 @@
       <c r="I279" s="7">
         <v>37</v>
       </c>
-      <c r="J279" s="8"/>
-      <c r="K279" s="8"/>
-      <c r="L279" s="8"/>
-      <c r="M279" s="8"/>
+      <c r="J279" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K279" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L279" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M279" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N279" s="5" t="s">
         <v>762</v>
       </c>
@@ -14151,10 +15673,18 @@
       <c r="I280" s="7">
         <v>95</v>
       </c>
-      <c r="J280" s="8"/>
-      <c r="K280" s="8"/>
-      <c r="L280" s="8"/>
-      <c r="M280" s="8"/>
+      <c r="J280" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K280" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L280" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M280" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N280" s="5" t="s">
         <v>766</v>
       </c>
@@ -14231,10 +15761,18 @@
       <c r="I282" s="7">
         <v>92</v>
       </c>
-      <c r="J282" s="8"/>
-      <c r="K282" s="8"/>
-      <c r="L282" s="8"/>
-      <c r="M282" s="8"/>
+      <c r="J282" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K282" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L282" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M282" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N282" s="5" t="s">
         <v>774</v>
       </c>
@@ -14267,10 +15805,18 @@
       <c r="I283" s="7">
         <v>124</v>
       </c>
-      <c r="J283" s="8"/>
-      <c r="K283" s="8"/>
-      <c r="L283" s="8"/>
-      <c r="M283" s="8"/>
+      <c r="J283" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K283" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L283" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M283" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N283" s="5" t="s">
         <v>778</v>
       </c>
@@ -14303,10 +15849,18 @@
       <c r="I284" s="7">
         <v>30</v>
       </c>
-      <c r="J284" s="8"/>
-      <c r="K284" s="8"/>
-      <c r="L284" s="8"/>
-      <c r="M284" s="8"/>
+      <c r="J284" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K284" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L284" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M284" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N284" s="5" t="s">
         <v>781</v>
       </c>
@@ -14339,10 +15893,18 @@
       <c r="I285" s="7">
         <v>21</v>
       </c>
-      <c r="J285" s="8"/>
-      <c r="K285" s="8"/>
-      <c r="L285" s="8"/>
-      <c r="M285" s="8"/>
+      <c r="J285" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K285" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L285" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M285" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N285" s="5" t="s">
         <v>785</v>
       </c>
@@ -14375,10 +15937,18 @@
       <c r="I286" s="7">
         <v>398</v>
       </c>
-      <c r="J286" s="8"/>
-      <c r="K286" s="8"/>
-      <c r="L286" s="8"/>
-      <c r="M286" s="8"/>
+      <c r="J286" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K286" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L286" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M286" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N286" s="5" t="s">
         <v>788</v>
       </c>
@@ -14411,10 +15981,18 @@
       <c r="I287" s="7">
         <v>14</v>
       </c>
-      <c r="J287" s="8"/>
-      <c r="K287" s="8"/>
-      <c r="L287" s="8"/>
-      <c r="M287" s="8"/>
+      <c r="J287" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="K287" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="L287" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="M287" s="8" t="s">
+        <v>13</v>
+      </c>
       <c r="N287" s="5" t="s">
         <v>791</v>
       </c>

</xml_diff>